<commit_message>
Name it the Global Database Format for Realtors
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RZ6ERERyGbK7VA7w662RHW
</commit_message>
<xml_diff>
--- a/public/listing-template.xlsx
+++ b/public/listing-template.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="4">
@@ -65,11 +69,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -700,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -709,77 +714,50 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Global Database Format for Realtors · sellmyhouse.asia</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Required?</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>What to put in it</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Asking price as a number. 450000, 450,000, RM 450,000 and 1.2m all work.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>currency</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>3-letter code: MYR, SGD, USD, GBP, EUR, AUD, THB… Read from the price if left blank (RM, S$, £, €).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>price</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Required*</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Town and country, e.g. Ipoh, Perak, Malaysia. *Or leave blank and fill latitude and longitude.</t>
+          <t>Asking price as a number. 450000, 450,000, RM 450,000 and 1.2m all work.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -789,48 +767,48 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Map pin, decimal degrees, e.g. 4.5975. Puts the listing on the exact spot on the world map.</t>
+          <t>3-letter code: MYR, SGD, USD, GBP, EUR, AUD, THB… Read from the price if left blank (RM, S$, £, €).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Required*</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Map pin, decimal degrees, e.g. 101.0901.</t>
+          <t>Town and country, e.g. Ipoh, Perak, Malaysia. *Or leave blank and fill latitude and longitude.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>contact_name</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Seller's or realtor's name, shown to buyers.</t>
+          <t>Map pin, decimal degrees, e.g. 4.5975. Puts the listing on the exact spot on the world map.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>contact_phone</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -840,31 +818,31 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>With country code if possible, e.g. +60 12 345 6789. Shown with Call and WhatsApp buttons.</t>
+          <t>Map pin, decimal degrees, e.g. 101.0901.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>contact_email</t>
+          <t>contact_name</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Shown with an Email button.</t>
+          <t>Seller's or realtor's name, shown to buyers.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>agency</t>
+          <t>contact_phone</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -874,14 +852,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Realtors only: your agency name. Leave blank for a private sale.</t>
+          <t>With country code if possible, e.g. +60 12 345 6789. Shown with Call and WhatsApp buttons.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>contact_email</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -891,14 +869,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Short headline. Left blank, we write one, e.g. 3-bedroom house in Ipoh.</t>
+          <t>Shown with an Email button.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>property_type</t>
+          <t>agency</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -908,14 +886,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>House, Condominium, Apartment, Terrace, Semi-detached, Bungalow, Villa, Townhouse, Land…</t>
+          <t>Realtors only: your agency name. Leave blank for a private sale.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>bedrooms</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -925,14 +903,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Whole number. Studio = 0.</t>
+          <t>Short headline. Left blank, we write one, e.g. 3-bedroom house in Ipoh.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>bathrooms</t>
+          <t>property_type</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -942,14 +920,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Whole number.</t>
+          <t>House, Condominium, Apartment, Terrace, Semi-detached, Bungalow, Villa, Townhouse, Land…</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>built_up</t>
+          <t>bedrooms</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -959,14 +937,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Floor area as a number. Units can go in the cell (1,200 sqft) or in area_unit.</t>
+          <t>Whole number. Studio = 0.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>land_size</t>
+          <t>bathrooms</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -976,14 +954,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Land or plot area as a number.</t>
+          <t>Whole number.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>area_unit</t>
+          <t>built_up</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -993,14 +971,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>sq ft, sq m, acres or hectares.</t>
+          <t>Floor area as a number. Units can go in the cell (1,200 sqft) or in area_unit.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>tenure</t>
+          <t>land_size</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1010,14 +988,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Freehold, Leasehold, or your local term (e.g. 99-year leasehold, Strata).</t>
+          <t>Land or plot area as a number.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>area_unit</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1027,14 +1005,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Up to 2,000 characters.</t>
+          <t>sq ft, sq m, acres or hectares.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>image_urls</t>
+          <t>tenure</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1044,14 +1022,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Up to 12 photo links (https://…), separated by spaces or |. Or use columns image_1, image_2…</t>
+          <t>Freehold, Leasehold, or your local term (e.g. 99-year leasehold, Strata).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1061,14 +1039,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Your own listing ID, so you can match listings back to your system.</t>
+          <t>Up to 2,000 characters.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>listing_url</t>
+          <t>image_urls</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1078,12 +1056,47 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Link to the listing on your own website.</t>
+          <t>Up to 12 photo links (https://…), separated by spaces or |. Or use columns image_1, image_2…</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Your own listing ID, so you can match listings back to your system.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
+        <is>
+          <t>listing_url</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Link to the listing on your own website.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Only price, location (or latitude + longitude) and contact_name are required. Fill the Listings sheet (one property per row), save, and upload at sellmyhouse.asia/upload. Up to 200 listings per file.</t>
         </is>
@@ -1251,8 +1264,6 @@
           <t>aisha@example.com</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>Terrace</t>
@@ -1273,7 +1284,6 @@
           <t>1650</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>sq ft</t>
@@ -1294,8 +1304,6 @@
           <t>https://example.com/photo1.jpg | https://example.com/photo2.jpg</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1308,7 +1316,6 @@
           <t>SGD</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>1.3521</t>
@@ -1329,7 +1336,6 @@
           <t>+65 9123 4567</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>Example Realty Pte Ltd</t>
@@ -1360,7 +1366,6 @@
           <t>850</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>sq ft</t>
@@ -1371,8 +1376,6 @@
           <t>99-year leasehold</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
           <t>ER-1042</t>
@@ -1390,27 +1393,21 @@
           <t>£325,000</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Bath, Somerset, United Kingdom</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Sarah Jones</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>sarah@example.com</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>Cottage</t>
@@ -1426,7 +1423,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
           <t>0.25</t>
@@ -1447,9 +1443,6 @@
           <t>Stone cottage with garden.</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Long-term rentals across the site
- 'Sell / Rent out' on the one-page form with deposit, furnishing,
  available-from and minimum lease; /sell?deal=rent preselects it
- Rentals stored in metadata (saleType rent), price is per month; shown
  as 'MYR 2,500 / month', 'For rent', with terms and a scam warning
- Buy / Rent / Both on search, rent price bands, Rent in the menu
- Both upload formats gain sale-or-rent and rental columns (generated by
  scripts/make-templates.py)
- Long-term only: minimum lease 6 months; short-stay listings refused
- For Rent signs; rentals compare with nearby rentals only

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RZ6ERERyGbK7VA7w662RHW
</commit_message>
<xml_diff>
--- a/public/listing-template.xlsx
+++ b/public/listing-template.xlsx
@@ -33,10 +33,10 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
-      <sz val="14"/>
     </font>
   </fonts>
   <fills count="4">
@@ -48,12 +48,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C2410C"/>
+        <fgColor rgb="003F3F46"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003F3F46"/>
+        <fgColor rgb="00C2410C"/>
       </patternFill>
     </fill>
   </fills>
@@ -159,105 +159,130 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Required. Asking price as a number. 450000, 450,000, RM 450,000 and 1.2m all work.</t>
+        <t>Optional. sale or rent. Blank means sale. Long-term rentals only: 6 months or more. No holiday lets or short stays.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. 3-letter code: MYR, SGD, USD, GBP, EUR, AUD, THB… Read from the price if left blank (RM, S$, £, €).</t>
+        <t>Required. Asking price, or the monthly rent for rentals. 450000, 450,000, RM 450,000 and 1.2m all work.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
+        <t>Optional. 3-letter code: MYR, SGD, USD, GBP, EUR, AUD, THB… Read from the price or location if left blank.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
         <t>Required*. Town and country, e.g. Ipoh, Perak, Malaysia. *Or leave blank and fill latitude and longitude.</t>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Map pin, decimal degrees, e.g. 4.5975. Puts the listing on the exact spot on the world map.</t>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Map pin, decimal degrees, e.g. 101.0901.</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Required. Seller's or realtor's name, shown to buyers.</t>
-      </text>
-    </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
+        <t>Required. Seller's, landlord's or realtor's name, shown to buyers and tenants.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
         <t>Optional. With country code if possible, e.g. +60 12 345 6789. Shown with Call and WhatsApp buttons.</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Shown with an Email button.</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Realtors only: your agency name. Leave blank for a private sale.</t>
-      </text>
-    </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
+        <t>Optional. Realtors only: your agency name. Leave blank for a private listing.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
         <t>Optional. Short headline. Left blank, we write one, e.g. 3-bedroom house in Ipoh.</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <t>Optional. House, Condominium, Apartment, Terrace, Semi-detached, Bungalow, Villa, Townhouse, Land…</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Whole number. Studio = 0.</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Whole number.</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Floor area as a number. Units can go in the cell (1,200 sqft) or in area_unit.</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Land or plot area as a number.</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <t>Optional. sq ft, sq m, acres or hectares.</t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Freehold, Leasehold, or your local term (e.g. 99-year leasehold, Strata).</t>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Rentals: the deposit amount.</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Rentals: Furnished, Partly furnished or Unfurnished.</t>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Rentals: a date (2026-12-01) or Now.</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Rentals: 6 or more.</t>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Up to 2,000 characters.</t>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Up to 12 photo links (https://…), separated by spaces or |. Or use columns image_1, image_2…</t>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Your own listing ID, so you can match listings back to your system.</t>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Link to the listing on your own website.</t>
       </text>
@@ -555,143 +580,179 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:Z1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="24" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="15" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>listing_type</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
           <t>price</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>latitude</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>longitude</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>contact_name</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>contact_phone</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>contact_email</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>agency</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>property_type</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>bedrooms</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>bathrooms</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>built_up</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>land_size</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>area_unit</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>tenure</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>deposit</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>furnished</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>available_from</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>minimum_lease_months</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>image_urls</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>reference</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>listing_url</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="P2:P1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="3">
+    <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"sale,rent"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q2:Q1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"sq ft,sq m,acres,hectares"</formula1>
+    </dataValidation>
+    <dataValidation sqref="T2:T1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Furnished,Partly furnished,Unfurnished"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -705,110 +766,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="110" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Global Database Format for Realtors · sellmyhouse.asia</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>One property per row on the Listings tab (only that tab is read). Save, then upload at sellmyhouse.asia/upload. Free, no account.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Long-term rentals only: 6 months or more. No holiday lets or short stays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Required?</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Needed?</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>What to put in it</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Asking price as a number. 450000, 450,000, RM 450,000 and 1.2m all work.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>currency</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>3-letter code: MYR, SGD, USD, GBP, EUR, AUD, THB… Read from the price if left blank (RM, S$, £, €).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>listing_type</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Required*</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Town and country, e.g. Ipoh, Perak, Malaysia. *Or leave blank and fill latitude and longitude.</t>
+          <t>sale or rent. Blank means sale. Long-term rentals only: 6 months or more. No holiday lets or short stays.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>price</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Map pin, decimal degrees, e.g. 4.5975. Puts the listing on the exact spot on the world map.</t>
+          <t>Asking price, or the monthly rent for rentals. 450000, 450,000, RM 450,000 and 1.2m all work.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -818,31 +859,31 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Map pin, decimal degrees, e.g. 101.0901.</t>
+          <t>3-letter code: MYR, SGD, USD, GBP, EUR, AUD, THB… Read from the price or location if left blank.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>contact_name</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Required*</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Seller's or realtor's name, shown to buyers.</t>
+          <t>Town and country, e.g. Ipoh, Perak, Malaysia. *Or leave blank and fill latitude and longitude.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>contact_phone</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -852,14 +893,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>With country code if possible, e.g. +60 12 345 6789. Shown with Call and WhatsApp buttons.</t>
+          <t>Map pin, decimal degrees, e.g. 4.5975. Puts the listing on the exact spot on the world map.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>contact_email</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -869,31 +910,31 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Shown with an Email button.</t>
+          <t>Map pin, decimal degrees, e.g. 101.0901.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>agency</t>
+          <t>contact_name</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Realtors only: your agency name. Leave blank for a private sale.</t>
+          <t>Seller's, landlord's or realtor's name, shown to buyers and tenants.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>contact_phone</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -903,14 +944,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Short headline. Left blank, we write one, e.g. 3-bedroom house in Ipoh.</t>
+          <t>With country code if possible, e.g. +60 12 345 6789. Shown with Call and WhatsApp buttons.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>property_type</t>
+          <t>contact_email</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -920,14 +961,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>House, Condominium, Apartment, Terrace, Semi-detached, Bungalow, Villa, Townhouse, Land…</t>
+          <t>Shown with an Email button.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>bedrooms</t>
+          <t>agency</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -937,14 +978,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Whole number. Studio = 0.</t>
+          <t>Realtors only: your agency name. Leave blank for a private listing.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>bathrooms</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -954,14 +995,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Whole number.</t>
+          <t>Short headline. Left blank, we write one, e.g. 3-bedroom house in Ipoh.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>built_up</t>
+          <t>property_type</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -971,14 +1012,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Floor area as a number. Units can go in the cell (1,200 sqft) or in area_unit.</t>
+          <t>House, Condominium, Apartment, Terrace, Semi-detached, Bungalow, Villa, Townhouse, Land…</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>land_size</t>
+          <t>bedrooms</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -988,14 +1029,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Land or plot area as a number.</t>
+          <t>Whole number. Studio = 0.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>area_unit</t>
+          <t>bathrooms</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1005,14 +1046,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>sq ft, sq m, acres or hectares.</t>
+          <t>Whole number.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>tenure</t>
+          <t>built_up</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1022,14 +1063,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Freehold, Leasehold, or your local term (e.g. 99-year leasehold, Strata).</t>
+          <t>Floor area as a number. Units can go in the cell (1,200 sqft) or in area_unit.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>land_size</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1039,14 +1080,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Up to 2,000 characters.</t>
+          <t>Land or plot area as a number.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>image_urls</t>
+          <t>area_unit</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1056,14 +1097,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Up to 12 photo links (https://…), separated by spaces or |. Or use columns image_1, image_2…</t>
+          <t>sq ft, sq m, acres or hectares.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>reference</t>
+          <t>tenure</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1073,14 +1114,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Your own listing ID, so you can match listings back to your system.</t>
+          <t>Freehold, Leasehold, or your local term (e.g. 99-year leasehold, Strata).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>listing_url</t>
+          <t>deposit</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1090,15 +1131,126 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Link to the listing on your own website.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
+          <t>Rentals: the deposit amount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>furnished</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Rentals: Furnished, Partly furnished or Unfurnished.</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Only price, location (or latitude + longitude) and contact_name are required. Fill the Listings sheet (one property per row), save, and upload at sellmyhouse.asia/upload. Up to 200 listings per file.</t>
+          <t>available_from</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Rentals: a date (2026-12-01) or Now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>minimum_lease_months</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Rentals: 6 or more.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Up to 2,000 characters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>image_urls</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Up to 12 photo links (https://…), separated by spaces or |. Or use columns image_1, image_2…</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Your own listing ID, so you can match listings back to your system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>listing_url</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Link to the listing on your own website.</t>
         </is>
       </c>
     </row>
@@ -1113,336 +1265,412 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:Z4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>listing_type</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>latitude</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>longitude</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>contact_name</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>contact_phone</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>contact_email</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>agency</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>property_type</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>bedrooms</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>bathrooms</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>built_up</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>land_size</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>area_unit</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>tenure</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>deposit</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>furnished</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>available_from</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>minimum_lease_months</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="X1" s="4" t="inlineStr">
         <is>
           <t>image_urls</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="Y1" s="4" t="inlineStr">
         <is>
           <t>reference</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>listing_url</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
         <is>
           <t>450000</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>MYR</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Ipoh, Perak, Malaysia</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>4.5975</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>101.0901</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Aisha Rahman</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>+60 12 345 6789</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>aisha@example.com</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
         <is>
           <t>Terrace</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>1650</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>sq ft</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Freehold</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
         <is>
           <t>Corner unit, renovated kitchen, near schools.</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>https://example.com/photo1.jpg | https://example.com/photo2.jpg</t>
         </is>
       </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1.2m</t>
+          <t>rent</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>3800</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>SGD</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
         <is>
           <t>1.3521</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>103.8198</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Daniel Tan</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>+65 9123 4567</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
         <is>
           <t>Example Realty Pte Ltd</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2-bedroom condo with pool view</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Condominium</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>850</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>sq ft</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>99-year leasehold</t>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>7600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
+          <t>Furnished</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr">
+        <is>
           <t>ER-1042</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>https://example.com/listings/1042</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
         <is>
           <t>£325,000</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Bath, Somerset, United Kingdom</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Sarah Jones</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
         <is>
           <t>sarah@example.com</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
         <is>
           <t>Cottage</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
         <is>
           <t>0.25</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>acres</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Freehold</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
         <is>
           <t>Stone cottage with garden.</t>
         </is>
       </c>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>